<commit_message>
Added config file and linked all tests to config. Removed redundant verify title test.
</commit_message>
<xml_diff>
--- a/test/test_resources/user_credentials.xlsx
+++ b/test/test_resources/user_credentials.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://akima365-my.sharepoint.com/personal/daniel_pearson_cloudlakellc_com/Documents/Desktop/Projects/MTT_4.0/test/test_resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="8_{1C1DD90D-7887-42B7-80F4-6722B28CE67C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{255777F3-EB83-4133-842C-31153B82EA9D}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="8_{1C1DD90D-7887-42B7-80F4-6722B28CE67C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE565F33-A8B0-4A21-B102-766468D46975}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{112304DE-681E-4BA1-800A-5CC861B4AC92}"/>
   </bookViews>
@@ -44,34 +44,26 @@
     <t>password</t>
   </si>
   <si>
-    <t>p@ssw0rd!</t>
-  </si>
-  <si>
     <t>bass079</t>
   </si>
   <si>
-    <t>Pearson</t>
-  </si>
-  <si>
     <t>Bass</t>
+  </si>
+  <si>
+    <t>pandearson</t>
+  </si>
+  <si>
+    <t>Khruangbin3@</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -94,16 +86,14 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -456,21 +446,18 @@
         <v>4</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{ECE25A20-613A-422B-9EE1-8C2B54882EEB}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Created python script file to run all tests for each browser separately and compile separate reports for each.
</commit_message>
<xml_diff>
--- a/test/test_resources/user_credentials.xlsx
+++ b/test/test_resources/user_credentials.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://akima365-my.sharepoint.com/personal/daniel_pearson_cloudlakellc_com/Documents/Desktop/Projects/MTT_4.0/test/test_resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="8_{1C1DD90D-7887-42B7-80F4-6722B28CE67C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE565F33-A8B0-4A21-B102-766468D46975}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="8_{1C1DD90D-7887-42B7-80F4-6722B28CE67C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{041B7A55-EB29-4E5F-BD14-0FE30429B6A0}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{112304DE-681E-4BA1-800A-5CC861B4AC92}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{112304DE-681E-4BA1-800A-5CC861B4AC92}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -50,10 +50,10 @@
     <t>Bass</t>
   </si>
   <si>
-    <t>pandearson</t>
-  </si>
-  <si>
-    <t>Khruangbin3@</t>
+    <t>Pearsond</t>
+  </si>
+  <si>
+    <t>P@ssw0rd!</t>
   </si>
 </sst>
 </file>
@@ -107,6 +107,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Updated script to be more accurate and open files accordingly.
</commit_message>
<xml_diff>
--- a/test/test_resources/user_credentials.xlsx
+++ b/test/test_resources/user_credentials.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://akima365-my.sharepoint.com/personal/daniel_pearson_cloudlakellc_com/Documents/Desktop/Projects/MTT_4.0/test/test_resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="8_{1C1DD90D-7887-42B7-80F4-6722B28CE67C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{041B7A55-EB29-4E5F-BD14-0FE30429B6A0}"/>
+  <xr:revisionPtr revIDLastSave="30" documentId="8_{1C1DD90D-7887-42B7-80F4-6722B28CE67C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7EFCF01-3E41-43CD-AE45-93511B9F08FB}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{112304DE-681E-4BA1-800A-5CC861B4AC92}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{112304DE-681E-4BA1-800A-5CC861B4AC92}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -50,10 +50,10 @@
     <t>Bass</t>
   </si>
   <si>
-    <t>Pearsond</t>
-  </si>
-  <si>
-    <t>P@ssw0rd!</t>
+    <t>Pearson</t>
+  </si>
+  <si>
+    <t>Khruangbin3@</t>
   </si>
 </sst>
 </file>

</xml_diff>